<commit_message>
Preserve named scalar blanks in SUMPRODUCT
</commit_message>
<xml_diff>
--- a/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/lookup-conformance-input.xlsx
+++ b/OfficeIMO.TestAssets/Documents/ExcelFormulaCorpus/lookup-conformance-input.xlsx
@@ -1,20 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:bookViews xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-    <x:workbookView/>
-  </x:bookViews>
-  <sheets>
-    <sheet name="Data" sheetId="1" r:id="rId1"/>
-    <sheet name="Report" sheetId="2" r:id="rId2"/>
-    <sheet name="Keys" sheetId="3" r:id="rId3"/>
-  </sheets>
-  <x:definedNames xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-    <x:definedName name="Calc">SUM(Data!$A$1:$A$6)*2</x:definedName>
-    <x:definedName name="Nested">Calc/2+1</x:definedName>
-    <x:definedName name="EmptyKey">'Keys'!$H$1</x:definedName>
-  </x:definedNames>
-</workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:bookViews>
+    <ns0:workbookView/>
+  </ns0:bookViews>
+  <ns0:sheets>
+    <ns0:sheet name="Data" sheetId="1" ns1:id="rId1"/>
+    <ns0:sheet name="Report" sheetId="2" ns1:id="rId2"/>
+    <ns0:sheet name="Keys" sheetId="3" ns1:id="rId3"/>
+  </ns0:sheets>
+  <ns0:definedNames>
+    <ns0:definedName name="Calc">SUM(Data!$A$1:$A$6)*2</ns0:definedName>
+    <ns0:definedName name="Nested">Calc/2+1</ns0:definedName>
+    <ns0:definedName name="EmptyKey">'Keys'!$H$1</ns0:definedName>
+    <ns0:definedName name="BlankExpression">IFERROR(Data!$F$5,77)</ns0:definedName>
+    <ns0:definedName name="BlankAlias">BlankExpression</ns0:definedName>
+    <ns0:definedName name="BlankReference">Data!$F$5</ns0:definedName>
+  </ns0:definedNames>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>